<commit_message>
Se modifica archivo Casos de prueba
</commit_message>
<xml_diff>
--- a/Casos de prueba.xlsx
+++ b/Casos de prueba.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="180">
   <si>
     <t>ID</t>
   </si>
@@ -527,55 +527,31 @@
     <t>Se sube la imágen pero hay un error en el banner que dice siguiente, pues no se ve el texto.</t>
   </si>
   <si>
-    <t>Cierre forzado (Crash) al intentar subir imagen con menos de 10MB de espacio disponible.</t>
-  </si>
-  <si>
-    <t>1. Abrir Instagram Lite. 2. Tocar el icono "+" para crear una nueva publicación. 3. Seleccionar cualquier imagen de la galería. 4. Tocar en "Siguiente" y luego en "Compartir".</t>
-  </si>
-  <si>
-    <t>La aplicación debe mostrar un mensaje de error amigable: "No hay suficiente espacio en el dispositivo para procesar la imagen" y permitir al usuario regresar al feed. En cambio la pantalla se queda en blanco por 3 segundos y aparece el mensaje de sistema: "Instagram Lite se detuvo".</t>
-  </si>
-  <si>
-    <t>Crítica (El usuario no puede usar la función principal y la app se rompe).</t>
-  </si>
-  <si>
-    <t>Bucle de carga infinita en la pestaña de Reels</t>
-  </si>
-  <si>
-    <t>1. Abrir la aplicación Instagram Lite. 2. Hacer clic en el icono central de Reels. 3. Deslizar hacia abajo rápidamente para pasar 5 o 6 videos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> - Esperado: El siguiente video debe precargarse y reproducirse fluidamente.
- - Obtenido: La pantalla se queda en negro con un círculo de carga infinito, incluso con una conexión Wi-Fi estable.</t>
-  </si>
-  <si>
-    <t>Media/Alta (Afecta el consumo de contenido principal)</t>
-  </si>
-  <si>
-    <t>Error de "Imagen no disponible" en Carruseles</t>
-  </si>
-  <si>
-    <t>1. Seleccionar una publicación que contenga un carrusel (múltiples fotos). 2. Deslizar hacia la derecha para ver la segunda o tercera imagen. 3. Regresar rápidamente a la primera imagen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> - Esperado: Todas las imágenes del carrusel deben ser visibles al deslizar.
- - Obtenido: Aparece un icono de "triángulo de advertencia" o un cuadro gris, indicando que la imagen no se pudo cargar.</t>
-  </si>
-  <si>
-    <t>Media (Impacta la experiencia visual pero no bloquea la app).</t>
-  </si>
-  <si>
-    <t>Cierre inesperado (Crash) al subir Stories con stickers</t>
-  </si>
-  <si>
-    <t>1. Tocar el icono de "+" para crear una Story. 2. Tomar una foto o subir una de la galería. 3. Intentar añadir un sticker interactivo (Encuesta, Enlace o Música).</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> - Esperado: El menú de stickers debe abrirse y permitir la selección.
- - Obtenido: La aplicación se congela por 2 segundos y se cierra inesperadamente, regresando al menú de inicio del teléfono.</t>
-  </si>
-  <si>
-    <t>Crítica (Interrumpe una función principal de creación).</t>
+    <t>Carpeta de evidencias CP_11</t>
+  </si>
+  <si>
+    <t>Notificación de solicitud de seguimiento aparece vacía</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click en el ícono de notificaciones. </t>
+  </si>
+  <si>
+    <t>Debe verse la cuenta que solicita ser agregada, pero no aparece nada y solo es posible verla al refrescar.</t>
+  </si>
+  <si>
+    <t>Carpeta de evidencias CP_30</t>
+  </si>
+  <si>
+    <t>Carga del feed con red 2G</t>
+  </si>
+  <si>
+    <t>1. Configurar red de navegación 2G en el dispositivo. 2. Ingresar a la aplicación. 3. Refrescar feed.</t>
+  </si>
+  <si>
+    <t>Debe verse el feed pero al ingresar a la aplicación no es posible ver nada y solo aparece que está cargando.</t>
+  </si>
+  <si>
+    <t>Carpeta de evidencias CP_32</t>
   </si>
 </sst>
 </file>
@@ -2312,7 +2288,9 @@
       <c r="D3" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="10"/>
+      <c r="E3" s="9" t="s">
+        <v>171</v>
+      </c>
       <c r="F3" s="10"/>
       <c r="G3" s="10"/>
       <c r="H3" s="10"/>
@@ -2336,19 +2314,21 @@
       <c r="Z3" s="10"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="B4" s="9" t="s">
+      <c r="A4" s="7" t="s">
         <v>172</v>
       </c>
+      <c r="B4" s="8" t="s">
+        <v>173</v>
+      </c>
       <c r="C4" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="E4" s="10"/>
+        <v>56</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>175</v>
+      </c>
       <c r="F4" s="10"/>
       <c r="G4" s="10"/>
       <c r="H4" s="10"/>
@@ -2372,57 +2352,99 @@
       <c r="Z4" s="10"/>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="B5" s="12" t="s">
+      <c r="A5" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="B5" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="C5" s="9" t="s">
         <v>178</v>
       </c>
+      <c r="D5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
+      <c r="W5" s="10"/>
+      <c r="X5" s="10"/>
+      <c r="Y5" s="10"/>
+      <c r="Z5" s="10"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>182</v>
-      </c>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="10"/>
+      <c r="S6" s="10"/>
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10"/>
+      <c r="W6" s="10"/>
+      <c r="X6" s="10"/>
+      <c r="Y6" s="10"/>
+      <c r="Z6" s="10"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>186</v>
-      </c>
+      <c r="A7" s="11"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8">
+      <c r="A8" s="14"/>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9">
-      <c r="A9" s="15"/>
+      <c r="A9" s="14"/>
       <c r="B9" s="12"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="14"/>
     </row>
     <row r="10">
-      <c r="B10" s="16"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="15"/>
+      <c r="B11" s="12"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="16"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>